<commit_message>
feat(users): assouplit l'import CSV utilisateurs et rend l'email optionnel
- import_csv générique : prénom/nom/matricule obligatoires, tout le reste
  optionnel (email, sexe, dates, contrat, coefficient, salaire, rôle,
  service/poste/site, N+1 par matricule) ; ajoute forfait_jour/tickets_restaurant,
  retire cadre de cet import
- email désormais nullable (email='' provoquait un conflit d'unicité dès le
  2e utilisateur sans email) ; imports Kostango/collaborateurs laissent
  l'email vide au lieu de générer un email factice
- retire complètement le champ categorie_socio_pro (modèle, admin, API,
  impression entretien, formulaire utilisateur)
- corrige plusieurs endroits frontend qui supposaient email toujours renseigné
- met à jour les templates xlsx d'import (colonnes brutes, sans commentaires),
  ajoute template_utilisateurs.xlsx pour le nouvel import générique
</commit_message>
<xml_diff>
--- a/doc/template_augmentations.xlsx
+++ b/doc/template_augmentations.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,66 +26,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00555555"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00333333"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00666666"/>
-      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F7FB"/>
-        <bgColor rgb="00F2F7FB"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -93,37 +45,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B0B0B0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00B0B0B0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B0B0B0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00B0B0B0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,110 +417,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Import augmentations</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Remplacer la ligne exemple par vos données. Conserver l'en-tête (ligne 4).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
           <t>Matricule</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Montant Augmentation</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>00000001</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>01/01/2025</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>1500.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Description des colonnes :</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Matricule</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Matricule du collaborateur</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Date</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Date d'effet (JJ/MM/AAAA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Montant Augmentation</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Montant en euros (point ou virgule)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>